<commit_message>
Updated JPN_grids_kan model - 2026-05-12 18:27
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA19D3F2-BEEC-44FD-ABE7-D885DFB4C83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{19499898-BD75-4738-B53A-CD4703188C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7E22CEB-CC61-4A8A-A475-0464A8BC7F71}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6249FAC8-C5E9-4CF0-A652-39E487C52938}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6410B5B0-3EFB-4494-99B9-391F45D18249}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4B796C3-5D99-4D8B-AEB9-B47D85714A9A}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-12 18:40
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19499898-BD75-4738-B53A-CD4703188C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9BB8C96-EF98-46E2-9D7F-060B9F1856CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6249FAC8-C5E9-4CF0-A652-39E487C52938}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{647859EF-4B72-4F0E-A26F-13B035B2133C}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4B796C3-5D99-4D8B-AEB9-B47D85714A9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834A5FF5-AD23-4447-9961-A8778BEE3820}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-13 15:56
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9BB8C96-EF98-46E2-9D7F-060B9F1856CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FE56AD3-85E1-40A7-B199-2120CC22CBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{647859EF-4B72-4F0E-A26F-13B035B2133C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B258F-F36C-47C3-AE9E-E0D99C1B7E0B}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834A5FF5-AD23-4447-9961-A8778BEE3820}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD44FC9C-D673-4509-A8CC-B1A294934DCB}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-13 17:01
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FE56AD3-85E1-40A7-B199-2120CC22CBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C33DEF48-0B6E-47C8-AC8B-B9A6EE3F54BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B258F-F36C-47C3-AE9E-E0D99C1B7E0B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B7FB954-8727-4E67-AC6E-05C8394EFD2D}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD44FC9C-D673-4509-A8CC-B1A294934DCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48315BB4-77B4-4D8E-98BF-1DFB81CE7534}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-13 18:55
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C33DEF48-0B6E-47C8-AC8B-B9A6EE3F54BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A123705-5668-40DF-83AB-E2D03EE6CF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B7FB954-8727-4E67-AC6E-05C8394EFD2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6833092-4A9D-4276-A300-AB96999383E8}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48315BB4-77B4-4D8E-98BF-1DFB81CE7534}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E33D5A-8E18-4D19-8F6B-BD17EE4EBC9D}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-14 15:19
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A123705-5668-40DF-83AB-E2D03EE6CF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{523164AC-15C9-475C-BE94-F6FF4DF79A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6833092-4A9D-4276-A300-AB96999383E8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488A6565-DF69-4D51-931A-AD259A20ACC9}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E33D5A-8E18-4D19-8F6B-BD17EE4EBC9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C14DA68-CD45-4EAA-8D75-FCA9E0EA7CC0}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-14 15:23
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{523164AC-15C9-475C-BE94-F6FF4DF79A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD2B23A7-854B-4611-A1B2-8C317AD180EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488A6565-DF69-4D51-931A-AD259A20ACC9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92FF41E5-6EC4-42DF-B4C2-66A6A8956030}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C14DA68-CD45-4EAA-8D75-FCA9E0EA7CC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C694E4B-3D1A-4954-8A05-F944BDCE55B1}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-14 15:33
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD2B23A7-854B-4611-A1B2-8C317AD180EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07157112-4488-440F-9477-3B9B2679D9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92FF41E5-6EC4-42DF-B4C2-66A6A8956030}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{515EB854-6769-4B08-812D-6BFABADB3FC2}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C694E4B-3D1A-4954-8A05-F944BDCE55B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8AC1AB6-F5BD-456C-B5A4-C41433FE8141}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids_kan model - 2026-05-14 15:41
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07157112-4488-440F-9477-3B9B2679D9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBBE92E7-59F6-4162-826C-9B7C7A836FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -4720,7 +4720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{515EB854-6769-4B08-812D-6BFABADB3FC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69E8BD5A-0AEA-4E13-BA03-25FFB6915E29}">
   <dimension ref="B9:H302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -32394,7 +32394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8AC1AB6-F5BD-456C-B5A4-C41433FE8141}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56B213F4-3058-4DD5-9528-A00D3211D390}">
   <dimension ref="B9:L302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>